<commit_message>
Relabel A122-A154 (filled down by mistake); check A112
</commit_message>
<xml_diff>
--- a/data/labels/arrangement_dev_main.xlsx
+++ b/data/labels/arrangement_dev_main.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1076" uniqueCount="439">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1079" uniqueCount="442">
   <si>
     <t>sample_id</t>
   </si>
@@ -631,6 +631,9 @@
     <t>Remote Construction Business Office / Management Consulting</t>
   </si>
   <si>
+    <t>Remote may describe the work arrangement, but the title is broad enough that it is not fully clear what it modifies.</t>
+  </si>
+  <si>
     <t>A128</t>
   </si>
   <si>
@@ -667,6 +670,9 @@
     <t>CPA for a Remote U.S. Small Business</t>
   </si>
   <si>
+    <t>Remote describes the business, not how the CPA must work.</t>
+  </si>
+  <si>
     <t>A134</t>
   </si>
   <si>
@@ -779,6 +785,9 @@
   </si>
   <si>
     <t>Tailscale Remote Access Setup</t>
+  </si>
+  <si>
+    <t>Remote access describes the technical setup, not the worker’s arrangement.</t>
   </si>
   <si>
     <t>A153</t>
@@ -3037,7 +3046,7 @@
         <v>8</v>
       </c>
       <c r="D83" s="4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E83" s="4" t="s">
         <v>11</v>
@@ -3204,13 +3213,13 @@
         <v>195</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D93" s="4" t="s">
         <v>8</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="94" ht="15.75" customHeight="1">
@@ -3227,7 +3236,7 @@
         <v>8</v>
       </c>
       <c r="E94" s="4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="95" ht="15.75" customHeight="1">
@@ -3244,7 +3253,7 @@
         <v>8</v>
       </c>
       <c r="E95" s="4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="96" ht="15.75" customHeight="1">
@@ -3272,7 +3281,7 @@
         <v>203</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D97" s="4" t="s">
         <v>8</v>
@@ -3289,27 +3298,30 @@
         <v>205</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D98" s="4" t="s">
         <v>8</v>
       </c>
       <c r="E98" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="F98" s="4" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="99" ht="15.75" customHeight="1">
       <c r="A99" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C99" s="4" t="s">
         <v>8</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E99" s="4" t="s">
         <v>8</v>
@@ -3317,16 +3329,16 @@
     </row>
     <row r="100" ht="15.75" customHeight="1">
       <c r="A100" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C100" s="4" t="s">
         <v>8</v>
       </c>
       <c r="D100" s="4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E100" s="4" t="s">
         <v>8</v>
@@ -3334,10 +3346,10 @@
     </row>
     <row r="101" ht="15.75" customHeight="1">
       <c r="A101" s="2" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C101" s="4" t="s">
         <v>8</v>
@@ -3351,10 +3363,10 @@
     </row>
     <row r="102" ht="15.75" customHeight="1">
       <c r="A102" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C102" s="4" t="s">
         <v>8</v>
@@ -3368,10 +3380,10 @@
     </row>
     <row r="103" ht="15.75" customHeight="1">
       <c r="A103" s="2" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C103" s="4" t="s">
         <v>8</v>
@@ -3380,15 +3392,15 @@
         <v>8</v>
       </c>
       <c r="E103" s="4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="104" ht="15.75" customHeight="1">
       <c r="A104" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C104" s="4" t="s">
         <v>8</v>
@@ -3398,14 +3410,17 @@
       </c>
       <c r="E104" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="F104" s="4" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="105" ht="15.75" customHeight="1">
       <c r="A105" s="2" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C105" s="4" t="s">
         <v>8</v>
@@ -3419,10 +3434,10 @@
     </row>
     <row r="106" ht="15.75" customHeight="1">
       <c r="A106" s="2" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C106" s="4" t="s">
         <v>8</v>
@@ -3436,10 +3451,10 @@
     </row>
     <row r="107" ht="15.75" customHeight="1">
       <c r="A107" s="2" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C107" s="4" t="s">
         <v>8</v>
@@ -3448,15 +3463,15 @@
         <v>8</v>
       </c>
       <c r="E107" s="4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="108" ht="15.75" customHeight="1">
       <c r="A108" s="2" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C108" s="4" t="s">
         <v>8</v>
@@ -3465,15 +3480,15 @@
         <v>8</v>
       </c>
       <c r="E108" s="4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="109" ht="15.75" customHeight="1">
       <c r="A109" s="2" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C109" s="4" t="s">
         <v>8</v>
@@ -3487,10 +3502,10 @@
     </row>
     <row r="110" ht="15.75" customHeight="1">
       <c r="A110" s="2" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C110" s="4" t="s">
         <v>8</v>
@@ -3499,21 +3514,21 @@
         <v>8</v>
       </c>
       <c r="E110" s="4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="111" ht="15.75" customHeight="1">
       <c r="A111" s="2" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C111" s="4" t="s">
         <v>8</v>
       </c>
       <c r="D111" s="4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E111" s="4" t="s">
         <v>8</v>
@@ -3521,16 +3536,16 @@
     </row>
     <row r="112" ht="15.75" customHeight="1">
       <c r="A112" s="2" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C112" s="4" t="s">
         <v>8</v>
       </c>
       <c r="D112" s="4" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="E112" s="4" t="s">
         <v>8</v>
@@ -3538,10 +3553,10 @@
     </row>
     <row r="113" ht="15.75" customHeight="1">
       <c r="A113" s="2" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C113" s="4" t="s">
         <v>8</v>
@@ -3555,10 +3570,10 @@
     </row>
     <row r="114" ht="15.75" customHeight="1">
       <c r="A114" s="2" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C114" s="4" t="s">
         <v>8</v>
@@ -3567,15 +3582,15 @@
         <v>8</v>
       </c>
       <c r="E114" s="4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="115" ht="15.75" customHeight="1">
       <c r="A115" s="2" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C115" s="4" t="s">
         <v>8</v>
@@ -3589,10 +3604,10 @@
     </row>
     <row r="116" ht="15.75" customHeight="1">
       <c r="A116" s="2" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C116" s="4" t="s">
         <v>8</v>
@@ -3606,10 +3621,10 @@
     </row>
     <row r="117" ht="15.75" customHeight="1">
       <c r="A117" s="2" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C117" s="4" t="s">
         <v>8</v>
@@ -3626,10 +3641,10 @@
     </row>
     <row r="118" ht="15.75" customHeight="1">
       <c r="A118" s="2" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="C118" s="4" t="s">
         <v>8</v>
@@ -3643,16 +3658,16 @@
     </row>
     <row r="119" ht="15.75" customHeight="1">
       <c r="A119" s="2" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C119" s="4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D119" s="4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E119" s="4" t="s">
         <v>8</v>
@@ -3660,13 +3675,13 @@
     </row>
     <row r="120" ht="15.75" customHeight="1">
       <c r="A120" s="2" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B120" s="3" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C120" s="4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D120" s="4" t="s">
         <v>8</v>
@@ -3677,13 +3692,13 @@
     </row>
     <row r="121" ht="15.75" customHeight="1">
       <c r="A121" s="2" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B121" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C121" s="4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D121" s="4" t="s">
         <v>8</v>
@@ -3694,16 +3709,16 @@
     </row>
     <row r="122" ht="15.75" customHeight="1">
       <c r="A122" s="2" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C122" s="4" t="s">
         <v>8</v>
       </c>
       <c r="D122" s="4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E122" s="4" t="s">
         <v>8</v>
@@ -3711,10 +3726,10 @@
     </row>
     <row r="123" ht="15.75" customHeight="1">
       <c r="A123" s="2" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C123" s="4" t="s">
         <v>8</v>
@@ -3724,14 +3739,17 @@
       </c>
       <c r="E123" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="F123" s="4" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="124" ht="15.75" customHeight="1">
       <c r="A124" s="2" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="B124" s="3" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="C124" s="4" t="s">
         <v>8</v>
@@ -3740,21 +3758,21 @@
         <v>8</v>
       </c>
       <c r="E124" s="4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="125" ht="15.75" customHeight="1">
       <c r="A125" s="2" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="B125" s="3" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="C125" s="4" t="s">
         <v>8</v>
       </c>
       <c r="D125" s="4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E125" s="4" t="s">
         <v>8</v>
@@ -3762,10 +3780,10 @@
     </row>
     <row r="126" ht="15.75" customHeight="1">
       <c r="A126" s="2" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="C126" s="4" t="s">
         <v>11</v>
@@ -3779,10 +3797,10 @@
     </row>
     <row r="127" ht="15.75" customHeight="1">
       <c r="A127" s="2" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="B127" s="3" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="C127" s="4" t="s">
         <v>8</v>
@@ -3796,10 +3814,10 @@
     </row>
     <row r="128" ht="15.75" customHeight="1">
       <c r="A128" s="2" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="B128" s="3" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="C128" s="4" t="s">
         <v>11</v>
@@ -3813,10 +3831,10 @@
     </row>
     <row r="129" ht="15.75" customHeight="1">
       <c r="A129" s="2" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="C129" s="4" t="s">
         <v>8</v>
@@ -3830,10 +3848,10 @@
     </row>
     <row r="130" ht="15.75" customHeight="1">
       <c r="A130" s="2" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="B130" s="3" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="C130" s="4" t="s">
         <v>8</v>
@@ -3847,10 +3865,10 @@
     </row>
     <row r="131" ht="15.75" customHeight="1">
       <c r="A131" s="2" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="B131" s="3" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="C131" s="4" t="s">
         <v>11</v>
@@ -3864,10 +3882,10 @@
     </row>
     <row r="132" ht="15.75" customHeight="1">
       <c r="A132" s="2" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="B132" s="3" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="C132" s="4" t="s">
         <v>11</v>
@@ -3881,10 +3899,10 @@
     </row>
     <row r="133" ht="15.75" customHeight="1">
       <c r="A133" s="2" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="B133" s="3" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="C133" s="4" t="s">
         <v>8</v>
@@ -3898,10 +3916,10 @@
     </row>
     <row r="134" ht="15.75" customHeight="1">
       <c r="A134" s="2" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="B134" s="3" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="C134" s="4" t="s">
         <v>11</v>
@@ -3915,10 +3933,10 @@
     </row>
     <row r="135" ht="15.75" customHeight="1">
       <c r="A135" s="2" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B135" s="3" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C135" s="4" t="s">
         <v>8</v>
@@ -3932,10 +3950,10 @@
     </row>
     <row r="136" ht="15.75" customHeight="1">
       <c r="A136" s="2" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="B136" s="3" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="C136" s="4" t="s">
         <v>8</v>
@@ -3949,10 +3967,10 @@
     </row>
     <row r="137" ht="15.75" customHeight="1">
       <c r="A137" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B137" s="3" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="C137" s="4" t="s">
         <v>11</v>
@@ -3966,10 +3984,10 @@
     </row>
     <row r="138" ht="15.75" customHeight="1">
       <c r="A138" s="2" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="B138" s="3" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="C138" s="4" t="s">
         <v>11</v>
@@ -3983,10 +4001,10 @@
     </row>
     <row r="139" ht="15.75" customHeight="1">
       <c r="A139" s="2" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="B139" s="3" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C139" s="4" t="s">
         <v>8</v>
@@ -4000,10 +4018,10 @@
     </row>
     <row r="140" ht="15.75" customHeight="1">
       <c r="A140" s="2" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="B140" s="3" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="C140" s="4" t="s">
         <v>11</v>
@@ -4017,10 +4035,10 @@
     </row>
     <row r="141" ht="15.75" customHeight="1">
       <c r="A141" s="2" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="B141" s="3" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="C141" s="4" t="s">
         <v>8</v>
@@ -4034,10 +4052,10 @@
     </row>
     <row r="142" ht="15.75" customHeight="1">
       <c r="A142" s="2" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="B142" s="3" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="C142" s="4" t="s">
         <v>11</v>
@@ -4051,10 +4069,10 @@
     </row>
     <row r="143" ht="15.75" customHeight="1">
       <c r="A143" s="2" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="B143" s="3" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="C143" s="4" t="s">
         <v>8</v>
@@ -4068,10 +4086,10 @@
     </row>
     <row r="144" ht="15.75" customHeight="1">
       <c r="A144" s="2" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="B144" s="3" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="C144" s="4" t="s">
         <v>8</v>
@@ -4085,10 +4103,10 @@
     </row>
     <row r="145" ht="15.75" customHeight="1">
       <c r="A145" s="2" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="B145" s="3" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="C145" s="4" t="s">
         <v>8</v>
@@ -4102,10 +4120,10 @@
     </row>
     <row r="146" ht="15.75" customHeight="1">
       <c r="A146" s="2" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="B146" s="3" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="C146" s="4" t="s">
         <v>8</v>
@@ -4119,10 +4137,10 @@
     </row>
     <row r="147" ht="15.75" customHeight="1">
       <c r="A147" s="2" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="B147" s="3" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="C147" s="4" t="s">
         <v>8</v>
@@ -4136,10 +4154,10 @@
     </row>
     <row r="148" ht="15.75" customHeight="1">
       <c r="A148" s="2" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="B148" s="3" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="C148" s="4" t="s">
         <v>8</v>
@@ -4153,10 +4171,10 @@
     </row>
     <row r="149" ht="15.75" customHeight="1">
       <c r="A149" s="2" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="B149" s="3" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="C149" s="4" t="s">
         <v>8</v>
@@ -4170,10 +4188,10 @@
     </row>
     <row r="150" ht="15.75" customHeight="1">
       <c r="A150" s="2" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B150" s="3" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="C150" s="4" t="s">
         <v>11</v>
@@ -4187,10 +4205,10 @@
     </row>
     <row r="151" ht="15.75" customHeight="1">
       <c r="A151" s="2" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B151" s="3" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="C151" s="4" t="s">
         <v>8</v>
@@ -4204,10 +4222,10 @@
     </row>
     <row r="152" ht="15.75" customHeight="1">
       <c r="A152" s="2" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="B152" s="3" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="C152" s="4" t="s">
         <v>8</v>
@@ -4221,10 +4239,10 @@
     </row>
     <row r="153" ht="15.75" customHeight="1">
       <c r="A153" s="2" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B153" s="3" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C153" s="4" t="s">
         <v>8</v>
@@ -4238,10 +4256,10 @@
     </row>
     <row r="154" ht="15.75" customHeight="1">
       <c r="A154" s="2" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B154" s="3" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="C154" s="4" t="s">
         <v>8</v>
@@ -4255,10 +4273,10 @@
     </row>
     <row r="155" ht="15.75" customHeight="1">
       <c r="A155" s="2" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B155" s="3" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="C155" s="4" t="s">
         <v>11</v>
@@ -4272,10 +4290,10 @@
     </row>
     <row r="156" ht="15.75" customHeight="1">
       <c r="A156" s="2" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B156" s="3" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="C156" s="4" t="s">
         <v>11</v>
@@ -4289,10 +4307,10 @@
     </row>
     <row r="157" ht="15.75" customHeight="1">
       <c r="A157" s="2" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B157" s="3" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="C157" s="4" t="s">
         <v>8</v>
@@ -4306,10 +4324,10 @@
     </row>
     <row r="158" ht="15.75" customHeight="1">
       <c r="A158" s="2" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="B158" s="3" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="C158" s="4" t="s">
         <v>8</v>
@@ -4323,10 +4341,10 @@
     </row>
     <row r="159" ht="15.75" customHeight="1">
       <c r="A159" s="2" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="B159" s="3" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="C159" s="4" t="s">
         <v>8</v>
@@ -4340,10 +4358,10 @@
     </row>
     <row r="160" ht="15.75" customHeight="1">
       <c r="A160" s="2" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="B160" s="3" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="C160" s="4" t="s">
         <v>8</v>
@@ -4360,10 +4378,10 @@
     </row>
     <row r="161" ht="15.75" customHeight="1">
       <c r="A161" s="2" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="B161" s="3" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="C161" s="4" t="s">
         <v>8</v>
@@ -4380,10 +4398,10 @@
     </row>
     <row r="162" ht="15.75" customHeight="1">
       <c r="A162" s="2" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="B162" s="3" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="C162" s="4" t="s">
         <v>8</v>
@@ -4397,10 +4415,10 @@
     </row>
     <row r="163" ht="15.75" customHeight="1">
       <c r="A163" s="2" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="B163" s="3" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="C163" s="4" t="s">
         <v>8</v>
@@ -4414,10 +4432,10 @@
     </row>
     <row r="164" ht="15.75" customHeight="1">
       <c r="A164" s="2" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="B164" s="3" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="C164" s="4" t="s">
         <v>8</v>
@@ -4431,10 +4449,10 @@
     </row>
     <row r="165" ht="15.75" customHeight="1">
       <c r="A165" s="2" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="B165" s="3" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="C165" s="4" t="s">
         <v>8</v>
@@ -4448,10 +4466,10 @@
     </row>
     <row r="166" ht="15.75" customHeight="1">
       <c r="A166" s="2" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="B166" s="3" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="C166" s="4" t="s">
         <v>11</v>
@@ -4465,10 +4483,10 @@
     </row>
     <row r="167" ht="15.75" customHeight="1">
       <c r="A167" s="2" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="B167" s="3" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="C167" s="4" t="s">
         <v>11</v>
@@ -4482,10 +4500,10 @@
     </row>
     <row r="168" ht="15.75" customHeight="1">
       <c r="A168" s="2" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="B168" s="3" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="C168" s="4" t="s">
         <v>8</v>
@@ -4499,10 +4517,10 @@
     </row>
     <row r="169" ht="15.75" customHeight="1">
       <c r="A169" s="2" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="B169" s="3" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="C169" s="4" t="s">
         <v>8</v>
@@ -4516,10 +4534,10 @@
     </row>
     <row r="170" ht="15.75" customHeight="1">
       <c r="A170" s="2" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="B170" s="3" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="C170" s="4" t="s">
         <v>8</v>
@@ -4533,10 +4551,10 @@
     </row>
     <row r="171" ht="15.75" customHeight="1">
       <c r="A171" s="2" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="B171" s="3" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="C171" s="4" t="s">
         <v>8</v>
@@ -4550,10 +4568,10 @@
     </row>
     <row r="172" ht="15.75" customHeight="1">
       <c r="A172" s="2" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="B172" s="3" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="C172" s="4" t="s">
         <v>8</v>
@@ -4567,10 +4585,10 @@
     </row>
     <row r="173" ht="15.75" customHeight="1">
       <c r="A173" s="2" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="B173" s="3" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="C173" s="4" t="s">
         <v>8</v>
@@ -4584,10 +4602,10 @@
     </row>
     <row r="174" ht="15.75" customHeight="1">
       <c r="A174" s="2" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="B174" s="3" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="C174" s="4" t="s">
         <v>8</v>
@@ -4601,10 +4619,10 @@
     </row>
     <row r="175" ht="15.75" customHeight="1">
       <c r="A175" s="2" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="B175" s="3" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="C175" s="4" t="s">
         <v>8</v>
@@ -4618,10 +4636,10 @@
     </row>
     <row r="176" ht="15.75" customHeight="1">
       <c r="A176" s="2" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="B176" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="C176" s="4" t="s">
         <v>8</v>
@@ -4635,10 +4653,10 @@
     </row>
     <row r="177" ht="15.75" customHeight="1">
       <c r="A177" s="2" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="B177" s="3" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="C177" s="4" t="s">
         <v>11</v>
@@ -4652,10 +4670,10 @@
     </row>
     <row r="178" ht="15.75" customHeight="1">
       <c r="A178" s="2" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="B178" s="3" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="C178" s="4" t="s">
         <v>8</v>
@@ -4669,10 +4687,10 @@
     </row>
     <row r="179" ht="15.75" customHeight="1">
       <c r="A179" s="2" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="B179" s="3" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="C179" s="4" t="s">
         <v>8</v>
@@ -4684,15 +4702,15 @@
         <v>8</v>
       </c>
       <c r="F179" s="4" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
     </row>
     <row r="180" ht="15.75" customHeight="1">
       <c r="A180" s="2" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="B180" s="3" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="C180" s="4" t="s">
         <v>8</v>
@@ -4706,10 +4724,10 @@
     </row>
     <row r="181" ht="15.75" customHeight="1">
       <c r="A181" s="2" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="B181" s="3" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="C181" s="4" t="s">
         <v>8</v>
@@ -4723,10 +4741,10 @@
     </row>
     <row r="182" ht="15.75" customHeight="1">
       <c r="A182" s="2" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="B182" s="3" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="C182" s="4" t="s">
         <v>8</v>
@@ -4743,10 +4761,10 @@
     </row>
     <row r="183" ht="15.75" customHeight="1">
       <c r="A183" s="2" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="B183" s="3" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="C183" s="4" t="s">
         <v>8</v>
@@ -4760,10 +4778,10 @@
     </row>
     <row r="184" ht="15.75" customHeight="1">
       <c r="A184" s="2" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="B184" s="3" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="C184" s="4" t="s">
         <v>8</v>
@@ -4777,10 +4795,10 @@
     </row>
     <row r="185" ht="15.75" customHeight="1">
       <c r="A185" s="2" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="B185" s="3" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="C185" s="4" t="s">
         <v>8</v>
@@ -4794,10 +4812,10 @@
     </row>
     <row r="186" ht="15.75" customHeight="1">
       <c r="A186" s="2" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="B186" s="3" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="C186" s="4" t="s">
         <v>8</v>
@@ -4811,10 +4829,10 @@
     </row>
     <row r="187" ht="15.75" customHeight="1">
       <c r="A187" s="2" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="B187" s="3" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="C187" s="4" t="s">
         <v>8</v>
@@ -4828,10 +4846,10 @@
     </row>
     <row r="188" ht="15.75" customHeight="1">
       <c r="A188" s="2" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="B188" s="3" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="C188" s="4" t="s">
         <v>8</v>
@@ -4845,10 +4863,10 @@
     </row>
     <row r="189" ht="15.75" customHeight="1">
       <c r="A189" s="2" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="B189" s="3" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="C189" s="4" t="s">
         <v>8</v>
@@ -4862,10 +4880,10 @@
     </row>
     <row r="190" ht="15.75" customHeight="1">
       <c r="A190" s="2" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="B190" s="3" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="C190" s="4" t="s">
         <v>8</v>
@@ -4879,10 +4897,10 @@
     </row>
     <row r="191" ht="15.75" customHeight="1">
       <c r="A191" s="2" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="B191" s="3" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="C191" s="4" t="s">
         <v>8</v>
@@ -4896,10 +4914,10 @@
     </row>
     <row r="192" ht="15.75" customHeight="1">
       <c r="A192" s="2" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="B192" s="3" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="C192" s="4" t="s">
         <v>8</v>
@@ -4913,10 +4931,10 @@
     </row>
     <row r="193" ht="15.75" customHeight="1">
       <c r="A193" s="2" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="B193" s="3" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="C193" s="4" t="s">
         <v>8</v>
@@ -4928,15 +4946,15 @@
         <v>8</v>
       </c>
       <c r="F193" s="4" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
     </row>
     <row r="194" ht="15.75" customHeight="1">
       <c r="A194" s="2" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="B194" s="3" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="C194" s="4" t="s">
         <v>8</v>
@@ -4950,10 +4968,10 @@
     </row>
     <row r="195" ht="15.75" customHeight="1">
       <c r="A195" s="2" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="B195" s="3" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="C195" s="4" t="s">
         <v>8</v>
@@ -4967,10 +4985,10 @@
     </row>
     <row r="196" ht="15.75" customHeight="1">
       <c r="A196" s="2" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="B196" s="3" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="C196" s="4" t="s">
         <v>8</v>
@@ -4984,10 +5002,10 @@
     </row>
     <row r="197" ht="15.75" customHeight="1">
       <c r="A197" s="2" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="B197" s="3" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="C197" s="4" t="s">
         <v>8</v>
@@ -5001,10 +5019,10 @@
     </row>
     <row r="198" ht="15.75" customHeight="1">
       <c r="A198" s="2" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="B198" s="3" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="C198" s="4" t="s">
         <v>8</v>
@@ -5016,15 +5034,15 @@
         <v>8</v>
       </c>
       <c r="F198" s="4" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
     </row>
     <row r="199" ht="15.75" customHeight="1">
       <c r="A199" s="2" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="B199" s="3" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="C199" s="4" t="s">
         <v>11</v>
@@ -5038,10 +5056,10 @@
     </row>
     <row r="200" ht="15.75" customHeight="1">
       <c r="A200" s="2" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="B200" s="3" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="C200" s="4" t="s">
         <v>8</v>
@@ -5055,10 +5073,10 @@
     </row>
     <row r="201" ht="15.75" customHeight="1">
       <c r="A201" s="2" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="B201" s="3" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="C201" s="4" t="s">
         <v>8</v>
@@ -5072,10 +5090,10 @@
     </row>
     <row r="202" ht="15.75" customHeight="1">
       <c r="A202" s="2" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="B202" s="3" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="C202" s="4" t="s">
         <v>11</v>
@@ -5089,10 +5107,10 @@
     </row>
     <row r="203" ht="15.75" customHeight="1">
       <c r="A203" s="2" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="B203" s="3" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="C203" s="4" t="s">
         <v>11</v>
@@ -5106,10 +5124,10 @@
     </row>
     <row r="204" ht="15.75" customHeight="1">
       <c r="A204" s="2" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="B204" s="3" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="C204" s="4" t="s">
         <v>8</v>
@@ -5123,10 +5141,10 @@
     </row>
     <row r="205" ht="15.75" customHeight="1">
       <c r="A205" s="2" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="B205" s="3" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="C205" s="4" t="s">
         <v>8</v>
@@ -5140,10 +5158,10 @@
     </row>
     <row r="206" ht="15.75" customHeight="1">
       <c r="A206" s="2" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="B206" s="3" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="C206" s="4" t="s">
         <v>8</v>
@@ -5157,10 +5175,10 @@
     </row>
     <row r="207" ht="15.75" customHeight="1">
       <c r="A207" s="2" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="B207" s="3" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="C207" s="4" t="s">
         <v>8</v>
@@ -5174,10 +5192,10 @@
     </row>
     <row r="208" ht="15.75" customHeight="1">
       <c r="A208" s="2" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="B208" s="3" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="C208" s="4" t="s">
         <v>8</v>
@@ -5191,10 +5209,10 @@
     </row>
     <row r="209" ht="15.75" customHeight="1">
       <c r="A209" s="2" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="B209" s="3" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="C209" s="4" t="s">
         <v>8</v>
@@ -5208,10 +5226,10 @@
     </row>
     <row r="210" ht="15.75" customHeight="1">
       <c r="A210" s="2" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="B210" s="3" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="C210" s="4" t="s">
         <v>11</v>
@@ -5225,10 +5243,10 @@
     </row>
     <row r="211" ht="15.75" customHeight="1">
       <c r="A211" s="2" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="B211" s="3" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="C211" s="4" t="s">
         <v>11</v>
@@ -5242,10 +5260,10 @@
     </row>
     <row r="212" ht="15.75" customHeight="1">
       <c r="A212" s="2" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="B212" s="3" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="C212" s="4" t="s">
         <v>8</v>
@@ -5259,10 +5277,10 @@
     </row>
     <row r="213" ht="15.75" customHeight="1">
       <c r="A213" s="2" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="B213" s="3" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="C213" s="4" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
Arrangement rules 1.0, evaluation quarantine, D-041 rules record; A192 relabelled
</commit_message>
<xml_diff>
--- a/data/labels/arrangement_dev_main.xlsx
+++ b/data/labels/arrangement_dev_main.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1079" uniqueCount="442">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1082" uniqueCount="445">
   <si>
     <t>sample_id</t>
   </si>
@@ -133,6 +133,9 @@
     <t>Hungarian to English translation for delivery tomorrow Mar 22 noon CET</t>
   </si>
   <si>
+    <t>CET only tells us the delivery time, not required working hours.</t>
+  </si>
+  <si>
     <t>A046</t>
   </si>
   <si>
@@ -583,6 +586,9 @@
     <t>by 4:30pm GMT - Remove the long pause from the recorded powerpoint presentation</t>
   </si>
   <si>
+    <t>GMT only tells us the delivery time, not required working hours.</t>
+  </si>
+  <si>
     <t>A120</t>
   </si>
   <si>
@@ -1028,6 +1034,9 @@
   </si>
   <si>
     <t>Shopify store with 6,000-8,000 products from in person store</t>
+  </si>
+  <si>
+    <t>In person store describes the store, not where the work happens.</t>
   </si>
   <si>
     <t>A193</t>
@@ -1904,15 +1913,18 @@
         <v>8</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>11</v>
+        <v>8</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>8</v>
@@ -1926,10 +1938,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>14</v>
@@ -1941,15 +1953,15 @@
         <v>8</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>8</v>
@@ -1963,10 +1975,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>8</v>
@@ -1980,10 +1992,10 @@
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>8</v>
@@ -1997,10 +2009,10 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>11</v>
@@ -2012,15 +2024,15 @@
         <v>8</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>8</v>
@@ -2034,10 +2046,10 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>8</v>
@@ -2051,10 +2063,10 @@
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>8</v>
@@ -2068,10 +2080,10 @@
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>11</v>
@@ -2085,10 +2097,10 @@
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>11</v>
@@ -2102,10 +2114,10 @@
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>8</v>
@@ -2119,10 +2131,10 @@
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>8</v>
@@ -2136,10 +2148,10 @@
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>8</v>
@@ -2153,10 +2165,10 @@
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>8</v>
@@ -2170,10 +2182,10 @@
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>8</v>
@@ -2187,10 +2199,10 @@
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C33" s="4" t="s">
         <v>8</v>
@@ -2204,10 +2216,10 @@
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C34" s="4" t="s">
         <v>8</v>
@@ -2221,10 +2233,10 @@
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C35" s="4" t="s">
         <v>8</v>
@@ -2238,10 +2250,10 @@
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>8</v>
@@ -2255,10 +2267,10 @@
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C37" s="4" t="s">
         <v>8</v>
@@ -2272,10 +2284,10 @@
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>8</v>
@@ -2284,15 +2296,15 @@
         <v>8</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>8</v>
@@ -2306,10 +2318,10 @@
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>8</v>
@@ -2323,10 +2335,10 @@
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>8</v>
@@ -2340,10 +2352,10 @@
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>11</v>
@@ -2357,10 +2369,10 @@
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C43" s="4" t="s">
         <v>11</v>
@@ -2374,10 +2386,10 @@
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>11</v>
@@ -2391,10 +2403,10 @@
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C45" s="4" t="s">
         <v>8</v>
@@ -2408,10 +2420,10 @@
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C46" s="4" t="s">
         <v>8</v>
@@ -2425,10 +2437,10 @@
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C47" s="4" t="s">
         <v>11</v>
@@ -2442,10 +2454,10 @@
     </row>
     <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C48" s="4" t="s">
         <v>8</v>
@@ -2459,10 +2471,10 @@
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C49" s="4" t="s">
         <v>11</v>
@@ -2476,10 +2488,10 @@
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C50" s="4" t="s">
         <v>8</v>
@@ -2493,10 +2505,10 @@
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C51" s="4" t="s">
         <v>8</v>
@@ -2510,10 +2522,10 @@
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C52" s="4" t="s">
         <v>8</v>
@@ -2527,10 +2539,10 @@
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C53" s="4" t="s">
         <v>8</v>
@@ -2544,10 +2556,10 @@
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C54" s="4" t="s">
         <v>11</v>
@@ -2561,10 +2573,10 @@
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C55" s="4" t="s">
         <v>8</v>
@@ -2578,10 +2590,10 @@
     </row>
     <row r="56" ht="15.75" customHeight="1">
       <c r="A56" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C56" s="4" t="s">
         <v>8</v>
@@ -2595,10 +2607,10 @@
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C57" s="4" t="s">
         <v>8</v>
@@ -2612,10 +2624,10 @@
     </row>
     <row r="58" ht="15.75" customHeight="1">
       <c r="A58" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C58" s="4" t="s">
         <v>8</v>
@@ -2629,10 +2641,10 @@
     </row>
     <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C59" s="4" t="s">
         <v>11</v>
@@ -2646,10 +2658,10 @@
     </row>
     <row r="60" ht="15.75" customHeight="1">
       <c r="A60" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C60" s="4" t="s">
         <v>8</v>
@@ -2663,10 +2675,10 @@
     </row>
     <row r="61" ht="15.75" customHeight="1">
       <c r="A61" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C61" s="4" t="s">
         <v>8</v>
@@ -2680,10 +2692,10 @@
     </row>
     <row r="62" ht="15.75" customHeight="1">
       <c r="A62" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C62" s="4" t="s">
         <v>8</v>
@@ -2697,10 +2709,10 @@
     </row>
     <row r="63" ht="15.75" customHeight="1">
       <c r="A63" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C63" s="4" t="s">
         <v>11</v>
@@ -2714,10 +2726,10 @@
     </row>
     <row r="64" ht="15.75" customHeight="1">
       <c r="A64" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C64" s="4" t="s">
         <v>8</v>
@@ -2731,10 +2743,10 @@
     </row>
     <row r="65" ht="15.75" customHeight="1">
       <c r="A65" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C65" s="4" t="s">
         <v>11</v>
@@ -2748,10 +2760,10 @@
     </row>
     <row r="66" ht="15.75" customHeight="1">
       <c r="A66" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C66" s="4" t="s">
         <v>8</v>
@@ -2765,10 +2777,10 @@
     </row>
     <row r="67" ht="15.75" customHeight="1">
       <c r="A67" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C67" s="4" t="s">
         <v>8</v>
@@ -2782,10 +2794,10 @@
     </row>
     <row r="68" ht="15.75" customHeight="1">
       <c r="A68" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C68" s="4" t="s">
         <v>11</v>
@@ -2799,10 +2811,10 @@
     </row>
     <row r="69" ht="15.75" customHeight="1">
       <c r="A69" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C69" s="4" t="s">
         <v>11</v>
@@ -2816,10 +2828,10 @@
     </row>
     <row r="70" ht="15.75" customHeight="1">
       <c r="A70" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C70" s="4" t="s">
         <v>8</v>
@@ -2833,10 +2845,10 @@
     </row>
     <row r="71" ht="15.75" customHeight="1">
       <c r="A71" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C71" s="4" t="s">
         <v>8</v>
@@ -2850,10 +2862,10 @@
     </row>
     <row r="72" ht="15.75" customHeight="1">
       <c r="A72" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C72" s="4" t="s">
         <v>8</v>
@@ -2867,10 +2879,10 @@
     </row>
     <row r="73" ht="15.75" customHeight="1">
       <c r="A73" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C73" s="4" t="s">
         <v>8</v>
@@ -2884,10 +2896,10 @@
     </row>
     <row r="74" ht="15.75" customHeight="1">
       <c r="A74" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C74" s="4" t="s">
         <v>8</v>
@@ -2901,10 +2913,10 @@
     </row>
     <row r="75" ht="15.75" customHeight="1">
       <c r="A75" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C75" s="4" t="s">
         <v>11</v>
@@ -2918,10 +2930,10 @@
     </row>
     <row r="76" ht="15.75" customHeight="1">
       <c r="A76" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C76" s="4" t="s">
         <v>11</v>
@@ -2935,10 +2947,10 @@
     </row>
     <row r="77" ht="15.75" customHeight="1">
       <c r="A77" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C77" s="4" t="s">
         <v>8</v>
@@ -2952,10 +2964,10 @@
     </row>
     <row r="78" ht="15.75" customHeight="1">
       <c r="A78" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C78" s="4" t="s">
         <v>8</v>
@@ -2969,10 +2981,10 @@
     </row>
     <row r="79" ht="15.75" customHeight="1">
       <c r="A79" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C79" s="4" t="s">
         <v>11</v>
@@ -2986,10 +2998,10 @@
     </row>
     <row r="80" ht="15.75" customHeight="1">
       <c r="A80" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C80" s="4" t="s">
         <v>8</v>
@@ -3003,10 +3015,10 @@
     </row>
     <row r="81" ht="15.75" customHeight="1">
       <c r="A81" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C81" s="4" t="s">
         <v>11</v>
@@ -3020,10 +3032,10 @@
     </row>
     <row r="82" ht="15.75" customHeight="1">
       <c r="A82" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C82" s="4" t="s">
         <v>8</v>
@@ -3037,10 +3049,10 @@
     </row>
     <row r="83" ht="15.75" customHeight="1">
       <c r="A83" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C83" s="4" t="s">
         <v>8</v>
@@ -3054,10 +3066,10 @@
     </row>
     <row r="84" ht="15.75" customHeight="1">
       <c r="A84" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C84" s="4" t="s">
         <v>8</v>
@@ -3071,10 +3083,10 @@
     </row>
     <row r="85" ht="15.75" customHeight="1">
       <c r="A85" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C85" s="4" t="s">
         <v>11</v>
@@ -3088,10 +3100,10 @@
     </row>
     <row r="86" ht="15.75" customHeight="1">
       <c r="A86" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C86" s="4" t="s">
         <v>8</v>
@@ -3105,10 +3117,10 @@
     </row>
     <row r="87" ht="15.75" customHeight="1">
       <c r="A87" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C87" s="4" t="s">
         <v>8</v>
@@ -3122,10 +3134,10 @@
     </row>
     <row r="88" ht="15.75" customHeight="1">
       <c r="A88" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C88" s="4" t="s">
         <v>8</v>
@@ -3139,10 +3151,10 @@
     </row>
     <row r="89" ht="15.75" customHeight="1">
       <c r="A89" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C89" s="4" t="s">
         <v>8</v>
@@ -3156,10 +3168,10 @@
     </row>
     <row r="90" ht="15.75" customHeight="1">
       <c r="A90" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C90" s="4" t="s">
         <v>8</v>
@@ -3168,15 +3180,18 @@
         <v>8</v>
       </c>
       <c r="E90" s="4" t="s">
-        <v>11</v>
+        <v>8</v>
+      </c>
+      <c r="F90" s="4" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="91" ht="15.75" customHeight="1">
       <c r="A91" s="2" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C91" s="4" t="s">
         <v>8</v>
@@ -3190,10 +3205,10 @@
     </row>
     <row r="92" ht="15.75" customHeight="1">
       <c r="A92" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C92" s="4" t="s">
         <v>11</v>
@@ -3207,10 +3222,10 @@
     </row>
     <row r="93" ht="15.75" customHeight="1">
       <c r="A93" s="2" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C93" s="4" t="s">
         <v>11</v>
@@ -3224,10 +3239,10 @@
     </row>
     <row r="94" ht="15.75" customHeight="1">
       <c r="A94" s="2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C94" s="4" t="s">
         <v>8</v>
@@ -3241,10 +3256,10 @@
     </row>
     <row r="95" ht="15.75" customHeight="1">
       <c r="A95" s="2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C95" s="4" t="s">
         <v>8</v>
@@ -3258,10 +3273,10 @@
     </row>
     <row r="96" ht="15.75" customHeight="1">
       <c r="A96" s="2" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C96" s="4" t="s">
         <v>8</v>
@@ -3275,10 +3290,10 @@
     </row>
     <row r="97" ht="15.75" customHeight="1">
       <c r="A97" s="2" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C97" s="4" t="s">
         <v>11</v>
@@ -3292,10 +3307,10 @@
     </row>
     <row r="98" ht="15.75" customHeight="1">
       <c r="A98" s="2" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C98" s="4" t="s">
         <v>14</v>
@@ -3307,15 +3322,15 @@
         <v>8</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
     </row>
     <row r="99" ht="15.75" customHeight="1">
       <c r="A99" s="2" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C99" s="4" t="s">
         <v>8</v>
@@ -3329,10 +3344,10 @@
     </row>
     <row r="100" ht="15.75" customHeight="1">
       <c r="A100" s="2" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C100" s="4" t="s">
         <v>8</v>
@@ -3346,10 +3361,10 @@
     </row>
     <row r="101" ht="15.75" customHeight="1">
       <c r="A101" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C101" s="4" t="s">
         <v>8</v>
@@ -3363,10 +3378,10 @@
     </row>
     <row r="102" ht="15.75" customHeight="1">
       <c r="A102" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C102" s="4" t="s">
         <v>8</v>
@@ -3380,10 +3395,10 @@
     </row>
     <row r="103" ht="15.75" customHeight="1">
       <c r="A103" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C103" s="4" t="s">
         <v>8</v>
@@ -3397,10 +3412,10 @@
     </row>
     <row r="104" ht="15.75" customHeight="1">
       <c r="A104" s="2" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C104" s="4" t="s">
         <v>8</v>
@@ -3412,15 +3427,15 @@
         <v>8</v>
       </c>
       <c r="F104" s="4" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="105" ht="15.75" customHeight="1">
       <c r="A105" s="2" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C105" s="4" t="s">
         <v>8</v>
@@ -3434,10 +3449,10 @@
     </row>
     <row r="106" ht="15.75" customHeight="1">
       <c r="A106" s="2" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C106" s="4" t="s">
         <v>8</v>
@@ -3451,10 +3466,10 @@
     </row>
     <row r="107" ht="15.75" customHeight="1">
       <c r="A107" s="2" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C107" s="4" t="s">
         <v>8</v>
@@ -3468,10 +3483,10 @@
     </row>
     <row r="108" ht="15.75" customHeight="1">
       <c r="A108" s="2" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C108" s="4" t="s">
         <v>8</v>
@@ -3485,10 +3500,10 @@
     </row>
     <row r="109" ht="15.75" customHeight="1">
       <c r="A109" s="2" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C109" s="4" t="s">
         <v>8</v>
@@ -3502,10 +3517,10 @@
     </row>
     <row r="110" ht="15.75" customHeight="1">
       <c r="A110" s="2" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C110" s="4" t="s">
         <v>8</v>
@@ -3519,10 +3534,10 @@
     </row>
     <row r="111" ht="15.75" customHeight="1">
       <c r="A111" s="2" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C111" s="4" t="s">
         <v>8</v>
@@ -3536,10 +3551,10 @@
     </row>
     <row r="112" ht="15.75" customHeight="1">
       <c r="A112" s="2" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C112" s="4" t="s">
         <v>8</v>
@@ -3553,10 +3568,10 @@
     </row>
     <row r="113" ht="15.75" customHeight="1">
       <c r="A113" s="2" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C113" s="4" t="s">
         <v>8</v>
@@ -3570,10 +3585,10 @@
     </row>
     <row r="114" ht="15.75" customHeight="1">
       <c r="A114" s="2" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C114" s="4" t="s">
         <v>8</v>
@@ -3587,10 +3602,10 @@
     </row>
     <row r="115" ht="15.75" customHeight="1">
       <c r="A115" s="2" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C115" s="4" t="s">
         <v>8</v>
@@ -3604,10 +3619,10 @@
     </row>
     <row r="116" ht="15.75" customHeight="1">
       <c r="A116" s="2" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C116" s="4" t="s">
         <v>8</v>
@@ -3621,10 +3636,10 @@
     </row>
     <row r="117" ht="15.75" customHeight="1">
       <c r="A117" s="2" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="C117" s="4" t="s">
         <v>8</v>
@@ -3641,10 +3656,10 @@
     </row>
     <row r="118" ht="15.75" customHeight="1">
       <c r="A118" s="2" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C118" s="4" t="s">
         <v>8</v>
@@ -3658,10 +3673,10 @@
     </row>
     <row r="119" ht="15.75" customHeight="1">
       <c r="A119" s="2" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C119" s="4" t="s">
         <v>11</v>
@@ -3675,10 +3690,10 @@
     </row>
     <row r="120" ht="15.75" customHeight="1">
       <c r="A120" s="2" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B120" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C120" s="4" t="s">
         <v>11</v>
@@ -3692,10 +3707,10 @@
     </row>
     <row r="121" ht="15.75" customHeight="1">
       <c r="A121" s="2" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B121" s="3" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C121" s="4" t="s">
         <v>11</v>
@@ -3709,10 +3724,10 @@
     </row>
     <row r="122" ht="15.75" customHeight="1">
       <c r="A122" s="2" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C122" s="4" t="s">
         <v>8</v>
@@ -3726,10 +3741,10 @@
     </row>
     <row r="123" ht="15.75" customHeight="1">
       <c r="A123" s="2" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C123" s="4" t="s">
         <v>8</v>
@@ -3741,15 +3756,15 @@
         <v>8</v>
       </c>
       <c r="F123" s="4" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="124" ht="15.75" customHeight="1">
       <c r="A124" s="2" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B124" s="3" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="C124" s="4" t="s">
         <v>8</v>
@@ -3763,10 +3778,10 @@
     </row>
     <row r="125" ht="15.75" customHeight="1">
       <c r="A125" s="2" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B125" s="3" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C125" s="4" t="s">
         <v>8</v>
@@ -3780,10 +3795,10 @@
     </row>
     <row r="126" ht="15.75" customHeight="1">
       <c r="A126" s="2" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C126" s="4" t="s">
         <v>11</v>
@@ -3797,10 +3812,10 @@
     </row>
     <row r="127" ht="15.75" customHeight="1">
       <c r="A127" s="2" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B127" s="3" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C127" s="4" t="s">
         <v>8</v>
@@ -3814,10 +3829,10 @@
     </row>
     <row r="128" ht="15.75" customHeight="1">
       <c r="A128" s="2" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B128" s="3" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C128" s="4" t="s">
         <v>11</v>
@@ -3831,10 +3846,10 @@
     </row>
     <row r="129" ht="15.75" customHeight="1">
       <c r="A129" s="2" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C129" s="4" t="s">
         <v>8</v>
@@ -3848,10 +3863,10 @@
     </row>
     <row r="130" ht="15.75" customHeight="1">
       <c r="A130" s="2" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B130" s="3" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C130" s="4" t="s">
         <v>8</v>
@@ -3865,10 +3880,10 @@
     </row>
     <row r="131" ht="15.75" customHeight="1">
       <c r="A131" s="2" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B131" s="3" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="C131" s="4" t="s">
         <v>11</v>
@@ -3882,10 +3897,10 @@
     </row>
     <row r="132" ht="15.75" customHeight="1">
       <c r="A132" s="2" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B132" s="3" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="C132" s="4" t="s">
         <v>11</v>
@@ -3899,10 +3914,10 @@
     </row>
     <row r="133" ht="15.75" customHeight="1">
       <c r="A133" s="2" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B133" s="3" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C133" s="4" t="s">
         <v>8</v>
@@ -3916,10 +3931,10 @@
     </row>
     <row r="134" ht="15.75" customHeight="1">
       <c r="A134" s="2" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B134" s="3" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C134" s="4" t="s">
         <v>11</v>
@@ -3933,10 +3948,10 @@
     </row>
     <row r="135" ht="15.75" customHeight="1">
       <c r="A135" s="2" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B135" s="3" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C135" s="4" t="s">
         <v>8</v>
@@ -3950,10 +3965,10 @@
     </row>
     <row r="136" ht="15.75" customHeight="1">
       <c r="A136" s="2" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B136" s="3" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C136" s="4" t="s">
         <v>8</v>
@@ -3967,10 +3982,10 @@
     </row>
     <row r="137" ht="15.75" customHeight="1">
       <c r="A137" s="2" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B137" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="C137" s="4" t="s">
         <v>11</v>
@@ -3984,10 +3999,10 @@
     </row>
     <row r="138" ht="15.75" customHeight="1">
       <c r="A138" s="2" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B138" s="3" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C138" s="4" t="s">
         <v>11</v>
@@ -4001,10 +4016,10 @@
     </row>
     <row r="139" ht="15.75" customHeight="1">
       <c r="A139" s="2" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B139" s="3" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C139" s="4" t="s">
         <v>8</v>
@@ -4018,10 +4033,10 @@
     </row>
     <row r="140" ht="15.75" customHeight="1">
       <c r="A140" s="2" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B140" s="3" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C140" s="4" t="s">
         <v>11</v>
@@ -4035,10 +4050,10 @@
     </row>
     <row r="141" ht="15.75" customHeight="1">
       <c r="A141" s="2" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B141" s="3" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="C141" s="4" t="s">
         <v>8</v>
@@ -4052,10 +4067,10 @@
     </row>
     <row r="142" ht="15.75" customHeight="1">
       <c r="A142" s="2" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B142" s="3" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C142" s="4" t="s">
         <v>11</v>
@@ -4069,10 +4084,10 @@
     </row>
     <row r="143" ht="15.75" customHeight="1">
       <c r="A143" s="2" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B143" s="3" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="C143" s="4" t="s">
         <v>8</v>
@@ -4086,10 +4101,10 @@
     </row>
     <row r="144" ht="15.75" customHeight="1">
       <c r="A144" s="2" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B144" s="3" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="C144" s="4" t="s">
         <v>8</v>
@@ -4103,10 +4118,10 @@
     </row>
     <row r="145" ht="15.75" customHeight="1">
       <c r="A145" s="2" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B145" s="3" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C145" s="4" t="s">
         <v>8</v>
@@ -4120,10 +4135,10 @@
     </row>
     <row r="146" ht="15.75" customHeight="1">
       <c r="A146" s="2" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B146" s="3" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="C146" s="4" t="s">
         <v>8</v>
@@ -4137,10 +4152,10 @@
     </row>
     <row r="147" ht="15.75" customHeight="1">
       <c r="A147" s="2" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B147" s="3" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="C147" s="4" t="s">
         <v>8</v>
@@ -4154,10 +4169,10 @@
     </row>
     <row r="148" ht="15.75" customHeight="1">
       <c r="A148" s="2" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B148" s="3" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="C148" s="4" t="s">
         <v>8</v>
@@ -4171,10 +4186,10 @@
     </row>
     <row r="149" ht="15.75" customHeight="1">
       <c r="A149" s="2" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B149" s="3" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="C149" s="4" t="s">
         <v>8</v>
@@ -4188,10 +4203,10 @@
     </row>
     <row r="150" ht="15.75" customHeight="1">
       <c r="A150" s="2" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B150" s="3" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="C150" s="4" t="s">
         <v>11</v>
@@ -4205,10 +4220,10 @@
     </row>
     <row r="151" ht="15.75" customHeight="1">
       <c r="A151" s="2" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B151" s="3" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="C151" s="4" t="s">
         <v>8</v>
@@ -4222,10 +4237,10 @@
     </row>
     <row r="152" ht="15.75" customHeight="1">
       <c r="A152" s="2" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B152" s="3" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="C152" s="4" t="s">
         <v>8</v>
@@ -4239,10 +4254,10 @@
     </row>
     <row r="153" ht="15.75" customHeight="1">
       <c r="A153" s="2" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B153" s="3" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C153" s="4" t="s">
         <v>8</v>
@@ -4256,10 +4271,10 @@
     </row>
     <row r="154" ht="15.75" customHeight="1">
       <c r="A154" s="2" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B154" s="3" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C154" s="4" t="s">
         <v>8</v>
@@ -4273,10 +4288,10 @@
     </row>
     <row r="155" ht="15.75" customHeight="1">
       <c r="A155" s="2" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B155" s="3" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="C155" s="4" t="s">
         <v>11</v>
@@ -4290,10 +4305,10 @@
     </row>
     <row r="156" ht="15.75" customHeight="1">
       <c r="A156" s="2" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B156" s="3" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C156" s="4" t="s">
         <v>11</v>
@@ -4307,10 +4322,10 @@
     </row>
     <row r="157" ht="15.75" customHeight="1">
       <c r="A157" s="2" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B157" s="3" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C157" s="4" t="s">
         <v>8</v>
@@ -4324,10 +4339,10 @@
     </row>
     <row r="158" ht="15.75" customHeight="1">
       <c r="A158" s="2" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B158" s="3" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C158" s="4" t="s">
         <v>8</v>
@@ -4341,10 +4356,10 @@
     </row>
     <row r="159" ht="15.75" customHeight="1">
       <c r="A159" s="2" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B159" s="3" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C159" s="4" t="s">
         <v>8</v>
@@ -4358,10 +4373,10 @@
     </row>
     <row r="160" ht="15.75" customHeight="1">
       <c r="A160" s="2" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B160" s="3" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="C160" s="4" t="s">
         <v>8</v>
@@ -4378,10 +4393,10 @@
     </row>
     <row r="161" ht="15.75" customHeight="1">
       <c r="A161" s="2" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B161" s="3" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="C161" s="4" t="s">
         <v>8</v>
@@ -4398,10 +4413,10 @@
     </row>
     <row r="162" ht="15.75" customHeight="1">
       <c r="A162" s="2" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B162" s="3" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="C162" s="4" t="s">
         <v>8</v>
@@ -4415,27 +4430,30 @@
     </row>
     <row r="163" ht="15.75" customHeight="1">
       <c r="A163" s="2" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B163" s="3" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="C163" s="4" t="s">
         <v>8</v>
       </c>
       <c r="D163" s="4" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E163" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="F163" s="4" t="s">
+        <v>341</v>
       </c>
     </row>
     <row r="164" ht="15.75" customHeight="1">
       <c r="A164" s="2" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="B164" s="3" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="C164" s="4" t="s">
         <v>8</v>
@@ -4449,10 +4467,10 @@
     </row>
     <row r="165" ht="15.75" customHeight="1">
       <c r="A165" s="2" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B165" s="3" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="C165" s="4" t="s">
         <v>8</v>
@@ -4466,10 +4484,10 @@
     </row>
     <row r="166" ht="15.75" customHeight="1">
       <c r="A166" s="2" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="B166" s="3" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="C166" s="4" t="s">
         <v>11</v>
@@ -4483,10 +4501,10 @@
     </row>
     <row r="167" ht="15.75" customHeight="1">
       <c r="A167" s="2" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="B167" s="3" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="C167" s="4" t="s">
         <v>11</v>
@@ -4500,10 +4518,10 @@
     </row>
     <row r="168" ht="15.75" customHeight="1">
       <c r="A168" s="2" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="B168" s="3" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="C168" s="4" t="s">
         <v>8</v>
@@ -4517,10 +4535,10 @@
     </row>
     <row r="169" ht="15.75" customHeight="1">
       <c r="A169" s="2" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="B169" s="3" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="C169" s="4" t="s">
         <v>8</v>
@@ -4534,10 +4552,10 @@
     </row>
     <row r="170" ht="15.75" customHeight="1">
       <c r="A170" s="2" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B170" s="3" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="C170" s="4" t="s">
         <v>8</v>
@@ -4551,10 +4569,10 @@
     </row>
     <row r="171" ht="15.75" customHeight="1">
       <c r="A171" s="2" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="B171" s="3" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="C171" s="4" t="s">
         <v>8</v>
@@ -4568,10 +4586,10 @@
     </row>
     <row r="172" ht="15.75" customHeight="1">
       <c r="A172" s="2" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="B172" s="3" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="C172" s="4" t="s">
         <v>8</v>
@@ -4585,10 +4603,10 @@
     </row>
     <row r="173" ht="15.75" customHeight="1">
       <c r="A173" s="2" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="B173" s="3" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="C173" s="4" t="s">
         <v>8</v>
@@ -4602,10 +4620,10 @@
     </row>
     <row r="174" ht="15.75" customHeight="1">
       <c r="A174" s="2" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="B174" s="3" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="C174" s="4" t="s">
         <v>8</v>
@@ -4619,10 +4637,10 @@
     </row>
     <row r="175" ht="15.75" customHeight="1">
       <c r="A175" s="2" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="B175" s="3" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="C175" s="4" t="s">
         <v>8</v>
@@ -4636,10 +4654,10 @@
     </row>
     <row r="176" ht="15.75" customHeight="1">
       <c r="A176" s="2" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="B176" s="3" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="C176" s="4" t="s">
         <v>8</v>
@@ -4653,10 +4671,10 @@
     </row>
     <row r="177" ht="15.75" customHeight="1">
       <c r="A177" s="2" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="B177" s="3" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="C177" s="4" t="s">
         <v>11</v>
@@ -4670,10 +4688,10 @@
     </row>
     <row r="178" ht="15.75" customHeight="1">
       <c r="A178" s="2" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="B178" s="3" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="C178" s="4" t="s">
         <v>8</v>
@@ -4687,10 +4705,10 @@
     </row>
     <row r="179" ht="15.75" customHeight="1">
       <c r="A179" s="2" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="B179" s="3" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="C179" s="4" t="s">
         <v>8</v>
@@ -4702,15 +4720,15 @@
         <v>8</v>
       </c>
       <c r="F179" s="4" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
     </row>
     <row r="180" ht="15.75" customHeight="1">
       <c r="A180" s="2" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="B180" s="3" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="C180" s="4" t="s">
         <v>8</v>
@@ -4724,10 +4742,10 @@
     </row>
     <row r="181" ht="15.75" customHeight="1">
       <c r="A181" s="2" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="B181" s="3" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="C181" s="4" t="s">
         <v>8</v>
@@ -4741,10 +4759,10 @@
     </row>
     <row r="182" ht="15.75" customHeight="1">
       <c r="A182" s="2" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="B182" s="3" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="C182" s="4" t="s">
         <v>8</v>
@@ -4761,10 +4779,10 @@
     </row>
     <row r="183" ht="15.75" customHeight="1">
       <c r="A183" s="2" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="B183" s="3" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="C183" s="4" t="s">
         <v>8</v>
@@ -4778,10 +4796,10 @@
     </row>
     <row r="184" ht="15.75" customHeight="1">
       <c r="A184" s="2" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="B184" s="3" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="C184" s="4" t="s">
         <v>8</v>
@@ -4795,10 +4813,10 @@
     </row>
     <row r="185" ht="15.75" customHeight="1">
       <c r="A185" s="2" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="B185" s="3" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="C185" s="4" t="s">
         <v>8</v>
@@ -4812,10 +4830,10 @@
     </row>
     <row r="186" ht="15.75" customHeight="1">
       <c r="A186" s="2" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="B186" s="3" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="C186" s="4" t="s">
         <v>8</v>
@@ -4829,10 +4847,10 @@
     </row>
     <row r="187" ht="15.75" customHeight="1">
       <c r="A187" s="2" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="B187" s="3" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="C187" s="4" t="s">
         <v>8</v>
@@ -4846,10 +4864,10 @@
     </row>
     <row r="188" ht="15.75" customHeight="1">
       <c r="A188" s="2" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="B188" s="3" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="C188" s="4" t="s">
         <v>8</v>
@@ -4863,10 +4881,10 @@
     </row>
     <row r="189" ht="15.75" customHeight="1">
       <c r="A189" s="2" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="B189" s="3" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="C189" s="4" t="s">
         <v>8</v>
@@ -4880,10 +4898,10 @@
     </row>
     <row r="190" ht="15.75" customHeight="1">
       <c r="A190" s="2" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B190" s="3" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="C190" s="4" t="s">
         <v>8</v>
@@ -4897,10 +4915,10 @@
     </row>
     <row r="191" ht="15.75" customHeight="1">
       <c r="A191" s="2" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="B191" s="3" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="C191" s="4" t="s">
         <v>8</v>
@@ -4914,10 +4932,10 @@
     </row>
     <row r="192" ht="15.75" customHeight="1">
       <c r="A192" s="2" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="B192" s="3" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="C192" s="4" t="s">
         <v>8</v>
@@ -4931,10 +4949,10 @@
     </row>
     <row r="193" ht="15.75" customHeight="1">
       <c r="A193" s="2" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="B193" s="3" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="C193" s="4" t="s">
         <v>8</v>
@@ -4946,15 +4964,15 @@
         <v>8</v>
       </c>
       <c r="F193" s="4" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
     </row>
     <row r="194" ht="15.75" customHeight="1">
       <c r="A194" s="2" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="B194" s="3" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="C194" s="4" t="s">
         <v>8</v>
@@ -4968,10 +4986,10 @@
     </row>
     <row r="195" ht="15.75" customHeight="1">
       <c r="A195" s="2" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="B195" s="3" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="C195" s="4" t="s">
         <v>8</v>
@@ -4985,10 +5003,10 @@
     </row>
     <row r="196" ht="15.75" customHeight="1">
       <c r="A196" s="2" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="B196" s="3" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="C196" s="4" t="s">
         <v>8</v>
@@ -5002,10 +5020,10 @@
     </row>
     <row r="197" ht="15.75" customHeight="1">
       <c r="A197" s="2" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="B197" s="3" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="C197" s="4" t="s">
         <v>8</v>
@@ -5019,10 +5037,10 @@
     </row>
     <row r="198" ht="15.75" customHeight="1">
       <c r="A198" s="2" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="B198" s="3" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="C198" s="4" t="s">
         <v>8</v>
@@ -5034,15 +5052,15 @@
         <v>8</v>
       </c>
       <c r="F198" s="4" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
     </row>
     <row r="199" ht="15.75" customHeight="1">
       <c r="A199" s="2" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="B199" s="3" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="C199" s="4" t="s">
         <v>11</v>
@@ -5056,10 +5074,10 @@
     </row>
     <row r="200" ht="15.75" customHeight="1">
       <c r="A200" s="2" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="B200" s="3" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="C200" s="4" t="s">
         <v>8</v>
@@ -5073,10 +5091,10 @@
     </row>
     <row r="201" ht="15.75" customHeight="1">
       <c r="A201" s="2" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="B201" s="3" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="C201" s="4" t="s">
         <v>8</v>
@@ -5090,10 +5108,10 @@
     </row>
     <row r="202" ht="15.75" customHeight="1">
       <c r="A202" s="2" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="B202" s="3" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="C202" s="4" t="s">
         <v>11</v>
@@ -5107,10 +5125,10 @@
     </row>
     <row r="203" ht="15.75" customHeight="1">
       <c r="A203" s="2" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="B203" s="3" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="C203" s="4" t="s">
         <v>11</v>
@@ -5124,10 +5142,10 @@
     </row>
     <row r="204" ht="15.75" customHeight="1">
       <c r="A204" s="2" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="B204" s="3" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="C204" s="4" t="s">
         <v>8</v>
@@ -5141,10 +5159,10 @@
     </row>
     <row r="205" ht="15.75" customHeight="1">
       <c r="A205" s="2" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="B205" s="3" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="C205" s="4" t="s">
         <v>8</v>
@@ -5158,10 +5176,10 @@
     </row>
     <row r="206" ht="15.75" customHeight="1">
       <c r="A206" s="2" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="B206" s="3" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="C206" s="4" t="s">
         <v>8</v>
@@ -5175,10 +5193,10 @@
     </row>
     <row r="207" ht="15.75" customHeight="1">
       <c r="A207" s="2" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="B207" s="3" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="C207" s="4" t="s">
         <v>8</v>
@@ -5192,10 +5210,10 @@
     </row>
     <row r="208" ht="15.75" customHeight="1">
       <c r="A208" s="2" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="B208" s="3" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="C208" s="4" t="s">
         <v>8</v>
@@ -5209,10 +5227,10 @@
     </row>
     <row r="209" ht="15.75" customHeight="1">
       <c r="A209" s="2" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="B209" s="3" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="C209" s="4" t="s">
         <v>8</v>
@@ -5226,10 +5244,10 @@
     </row>
     <row r="210" ht="15.75" customHeight="1">
       <c r="A210" s="2" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="B210" s="3" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="C210" s="4" t="s">
         <v>11</v>
@@ -5243,10 +5261,10 @@
     </row>
     <row r="211" ht="15.75" customHeight="1">
       <c r="A211" s="2" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="B211" s="3" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="C211" s="4" t="s">
         <v>11</v>
@@ -5260,10 +5278,10 @@
     </row>
     <row r="212" ht="15.75" customHeight="1">
       <c r="A212" s="2" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="B212" s="3" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="C212" s="4" t="s">
         <v>8</v>
@@ -5277,10 +5295,10 @@
     </row>
     <row r="213" ht="15.75" customHeight="1">
       <c r="A213" s="2" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="B213" s="3" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="C213" s="4" t="s">
         <v>11</v>

</xml_diff>